<commit_message>
Improved dashboard UI, export features and data manager fixes
</commit_message>
<xml_diff>
--- a/transactions.xlsx
+++ b/transactions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,72 +450,72 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Capital</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>450</v>
+        <v>100000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Burger-2</t>
+          <t>Business started</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Capital</t>
+          <t>Fuel</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>100000</v>
+        <v>5000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Business started</t>
+          <t>Bike</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fuel</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -524,17 +524,17 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>5000</v>
+        <v>25000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Bike</t>
+          <t>Rent paid</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -562,67 +562,67 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Rent</t>
+          <t xml:space="preserve">Land &amp; building </t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Expense</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>25000</v>
+        <v>100000</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Rent paid</t>
+          <t>Purchased</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Land &amp; building </t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Income</t>
+          <t>Expense</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>100000</v>
+        <v>2500</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Purchased</t>
+          <t>Biryani</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -636,26 +636,26 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Biryani</t>
+          <t>Cake</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t xml:space="preserve">Land purchase </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -664,26 +664,26 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>500</v>
+        <v>50000</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Cake</t>
+          <t xml:space="preserve">Purchase </t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Land purchase </t>
+          <t xml:space="preserve">Machinery </t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -692,17 +692,17 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>50000</v>
+        <v>25000</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Purchase </t>
+          <t>Purchased</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machinery </t>
+          <t>Machinery</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -725,6 +725,594 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>Purchased</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>24</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Land purchase</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Purchase</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>25</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>500</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Cake</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>26</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Biryani</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>27</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Land &amp; building</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Purchased</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>28</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Monthly salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>29</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Website project</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>30</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Office rent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>31</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Electricity</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>2400</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Electricity bill</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>32</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>999</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Broadband</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>33</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Fuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>34</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Stationery</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>650</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Office supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>35</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>27500</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Product sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>36</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Equipment repair</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>37</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Investment</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Dividend</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>38</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>6200</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Business trip</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>39</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Online ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>40</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Consulting fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>41</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Medical</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Clinic visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>42</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Performance bonus</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>43</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Miscellaneous</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>900</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Office snacks</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>44</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Rent paid</t>
         </is>
       </c>
     </row>

</xml_diff>